<commit_message>
Excel de control como fuente única y despliegue con ops.py
- config/control_plataforma.xlsx: parámetros, APIs, cuentas, permisos,
  usuarios, datasets, tablas, columnas y secretos; ops.py config genera
  tfvars, configuración y semillas de la API, con validación y --check en CI
- ops.py reemplaza Makefile/.env: bootstrap, plan, apply, datos, capas,
  api, verificar (BigQuery vs Excel), github, destroy, con log de tiempos
- Terraform parametrizado por el Excel; Cloud SQL, Cloud Run, WIF, DLQ
- Correcciones: publicadores esperan confirmación, Bronze con esquema
  explícito, Silver conserva fn/active, Gemini 3.1 Flash-Lite
- Documentos, matriz, calculadora y guía de despliegue actualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MgiFcvhexL3jkhqY5yJgLS
</commit_message>
<xml_diff>
--- a/docs/entrega1/Calculadora_Costos_GCP.xlsx
+++ b/docs/entrega1/Calculadora_Costos_GCP.xlsx
@@ -94,7 +94,7 @@
     <t xml:space="preserve">Serverless for Apache Spark</t>
   </si>
   <si>
-    <t xml:space="preserve">Vertex AI Gemini 2.5 Flash-Lite</t>
+    <t xml:space="preserve">Vertex AI Gemini 3.1 Flash-Lite</t>
   </si>
   <si>
     <t xml:space="preserve">Clave</t>
@@ -720,7 +720,7 @@
       </c>
       <c r="C3" s="2" t="n">
         <f aca="false">'Costo mensual'!C20</f>
-        <v>7.2</v>
+        <v>8.2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -729,7 +729,7 @@
       </c>
       <c r="C4" s="2" t="n">
         <f aca="false">'Costo mensual'!D20</f>
-        <v>9.72226</v>
+        <v>11.57226</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -738,7 +738,7 @@
       </c>
       <c r="C5" s="2" t="n">
         <f aca="false">'Costo mensual'!E20</f>
-        <v>281.82895</v>
+        <v>370.82895</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -747,7 +747,7 @@
       </c>
       <c r="C6" s="2" t="n">
         <f aca="false">'Costo mensual'!F20</f>
-        <v>958.2081</v>
+        <v>1403.2081</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -762,7 +762,7 @@
       </c>
       <c r="C8" s="4" t="n">
         <f aca="false">'Costo mensual'!E20*11+'Costo mensual'!F20*1</f>
-        <v>4058.32655</v>
+        <v>5482.32655</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -774,7 +774,7 @@
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">'Costo mensual'!C20*1+'Costo mensual'!D20*1</f>
-        <v>16.92226</v>
+        <v>19.77226</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -786,7 +786,7 @@
       </c>
       <c r="C11" s="5" t="n">
         <f aca="false">'Costo mensual'!E22</f>
-        <v>0.000747556896551724</v>
+        <v>0.000983631167108753</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -876,7 +876,7 @@
       </c>
       <c r="C22" s="2" t="n">
         <f aca="false">SUMIF('Costo mensual'!$B$2:$B$19,A22,'Costo mensual'!E$2:E$19)*11+SUMIF('Costo mensual'!$B$2:$B$19,A22,'Costo mensual'!F$2:F$19)*1</f>
-        <v>736</v>
+        <v>2160</v>
       </c>
     </row>
   </sheetData>
@@ -1234,7 +1234,7 @@
         <v>67</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="E17" s="6" t="n">
         <v>0</v>
@@ -1254,7 +1254,7 @@
         <v>70</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>0.4</v>
+        <v>1.5</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
@@ -2151,23 +2151,23 @@
       </c>
       <c r="B17" s="0" t="str">
         <f aca="false">Precios!B17</f>
-        <v>Vertex AI Gemini 2.5 Flash-Lite</v>
+        <v>Vertex AI Gemini 3.1 Flash-Lite</v>
       </c>
       <c r="C17" s="2" t="n">
         <f aca="false">MAX(0,Uso!C17-Precios!$E17)*Precios!$D17</f>
-        <v>0.3</v>
+        <v>0.75</v>
       </c>
       <c r="D17" s="2" t="n">
         <f aca="false">MAX(0,Uso!D17-Precios!$E17)*Precios!$D17</f>
-        <v>0.5</v>
+        <v>1.25</v>
       </c>
       <c r="E17" s="2" t="n">
         <f aca="false">MAX(0,Uso!E17-Precios!$E17)*Precios!$D17</f>
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="F17" s="2" t="n">
         <f aca="false">MAX(0,Uso!F17-Precios!$E17)*Precios!$D17</f>
-        <v>150</v>
+        <v>375</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2176,23 +2176,23 @@
       </c>
       <c r="B18" s="0" t="str">
         <f aca="false">Precios!B18</f>
-        <v>Vertex AI Gemini 2.5 Flash-Lite</v>
+        <v>Vertex AI Gemini 3.1 Flash-Lite</v>
       </c>
       <c r="C18" s="2" t="n">
         <f aca="false">MAX(0,Uso!C18-Precios!$E18)*Precios!$D18</f>
-        <v>0.2</v>
+        <v>0.75</v>
       </c>
       <c r="D18" s="2" t="n">
         <f aca="false">MAX(0,Uso!D18-Precios!$E18)*Precios!$D18</f>
-        <v>0.4</v>
+        <v>1.5</v>
       </c>
       <c r="E18" s="2" t="n">
         <f aca="false">MAX(0,Uso!E18-Precios!$E18)*Precios!$D18</f>
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="F18" s="2" t="n">
         <f aca="false">MAX(0,Uso!F18-Precios!$E18)*Precios!$D18</f>
-        <v>80</v>
+        <v>300</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2226,19 +2226,19 @@
       </c>
       <c r="C20" s="4" t="n">
         <f aca="false">SUM(C2:C19)</f>
-        <v>7.2</v>
+        <v>8.2</v>
       </c>
       <c r="D20" s="4" t="n">
         <f aca="false">SUM(D2:D19)</f>
-        <v>9.72226</v>
+        <v>11.57226</v>
       </c>
       <c r="E20" s="4" t="n">
         <f aca="false">SUM(E2:E19)</f>
-        <v>281.82895</v>
+        <v>370.82895</v>
       </c>
       <c r="F20" s="4" t="n">
         <f aca="false">SUM(F2:F19)</f>
-        <v>958.2081</v>
+        <v>1403.2081</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2268,19 +2268,19 @@
       </c>
       <c r="C22" s="10" t="n">
         <f aca="false">IF(C21&gt;0,C20/C21,0)</f>
-        <v>0.00144</v>
+        <v>0.00164</v>
       </c>
       <c r="D22" s="10" t="n">
         <f aca="false">IF(D21&gt;0,D20/D21,0)</f>
-        <v>0.000486113</v>
+        <v>0.000578613</v>
       </c>
       <c r="E22" s="10" t="n">
         <f aca="false">IF(E21&gt;0,E20/E21,0)</f>
-        <v>0.000747556896551724</v>
+        <v>0.000983631167108753</v>
       </c>
       <c r="F22" s="10" t="n">
         <f aca="false">IF(F21&gt;0,F20/F21,0)</f>
-        <v>0.000508333209549072</v>
+        <v>0.000744407480106101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>